<commit_message>
Fixed bidding calculation round one nafed
</commit_message>
<xml_diff>
--- a/testdata/BidDetailsData.xlsx.xlsx
+++ b/testdata/BidDetailsData.xlsx.xlsx
@@ -12,9 +12,9 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" fullCalcOnLoad="true"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -76,6 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="0"/>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -451,15 +452,15 @@
   <dimension ref="A1:AL4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="13.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="3" customWidth="1"/>
-    <col min="7" max="8" width="12" style="3" customWidth="1"/>
-    <col min="9" max="11" width="10.28515625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="3" customWidth="true" style="3" width="13.42578125"/>
+    <col min="4" max="4" customWidth="true" style="3" width="14.42578125"/>
+    <col min="5" max="5" customWidth="true" style="3" width="13.42578125"/>
+    <col min="6" max="6" customWidth="true" style="3" width="11.5703125"/>
+    <col min="7" max="8" customWidth="true" style="3" width="12.0"/>
+    <col min="9" max="11" customWidth="true" style="3" width="10.28515625"/>
+    <col min="12" max="12" customWidth="true" style="3" width="10.85546875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="3" width="11.28515625"/>
+    <col min="14" max="16384" style="3" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="90" x14ac:dyDescent="0.25">
@@ -526,34 +527,34 @@
       <c r="C2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="3">
-        <v>1828003460.03</v>
-      </c>
-      <c r="E2" s="3">
-        <v>13084425.689999999</v>
+      <c r="D2" s="3" t="n">
+        <v>1.82801076138E9</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1.307712434E7</v>
       </c>
       <c r="F2" s="3">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G2" s="3">
         <v>100</v>
       </c>
-      <c r="H2" s="3">
-        <v>58914.18</v>
-      </c>
-      <c r="I2" s="3">
-        <v>1828002956.53</v>
-      </c>
-      <c r="J2" s="3">
-        <v>13084929.189999999</v>
+      <c r="H2" s="3" t="n">
+        <v>60424.8</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>1.82795033658E9</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>1.313754914E7</v>
       </c>
       <c r="L2" s="3">
         <f>D2-I2</f>
-        <v>503.5</v>
+        <v>58914.200000047684</v>
       </c>
       <c r="M2" s="3">
         <f>J2-E2</f>
-        <v>503.5</v>
+        <v>58914.199999999255</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
@@ -589,34 +590,34 @@
       <c r="C3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3">
-        <v>168466040.02000001</v>
-      </c>
-      <c r="E3" s="3">
-        <v>10011197.880000001</v>
+      <c r="D3" s="3" t="n">
+        <v>1.6846604002E8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>1.001119788E7</v>
       </c>
       <c r="F3" s="3">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G3" s="3">
         <v>100</v>
       </c>
-      <c r="H3" s="3">
-        <v>58914.18</v>
-      </c>
-      <c r="I3" s="3">
-        <v>168406622.22</v>
-      </c>
-      <c r="J3" s="3">
-        <v>10070615.68</v>
+      <c r="H3" s="3" t="n">
+        <v>60928.34</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1.6840511172E8</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1.007212618E7</v>
       </c>
       <c r="L3" s="3">
         <f>D3-I3</f>
-        <v>59417.800000011921</v>
+        <v>59417.700000017881</v>
       </c>
       <c r="M3" s="3">
         <f>J3-E3</f>
-        <v>59417.799999998882</v>
+        <v>59417.699999999255</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.25">
@@ -629,34 +630,34 @@
       <c r="C4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3">
-        <v>1033142390.34</v>
-      </c>
-      <c r="E4" s="3">
-        <v>9016203.7200000007</v>
+      <c r="D4" s="3" t="n">
+        <v>1.03306508678E9</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9093507.28</v>
       </c>
       <c r="F4" s="3">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G4" s="3">
         <v>100</v>
       </c>
-      <c r="H4" s="3">
-        <v>58914.18</v>
-      </c>
-      <c r="I4" s="3">
-        <v>1033082469.04</v>
-      </c>
-      <c r="J4" s="3">
-        <v>9076125.0199999996</v>
+      <c r="H4" s="3" t="n">
+        <v>61431.88</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1.03300365488E9</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>9154939.18</v>
       </c>
       <c r="L4" s="3">
         <f>D4-I4</f>
-        <v>59921.300000071526</v>
+        <v>59921.299999952316</v>
       </c>
       <c r="M4" s="3">
         <f>J4-E4</f>
-        <v>59921.299999998882</v>
+        <v>59921.300000000745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
stable version for both catalog and bidding
</commit_message>
<xml_diff>
--- a/testdata/BidDetailsData.xlsx.xlsx
+++ b/testdata/BidDetailsData.xlsx.xlsx
@@ -534,27 +534,27 @@
         <v>1.307712434E7</v>
       </c>
       <c r="F2" s="3">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="G2" s="3">
         <v>100</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>60424.8</v>
+        <v>63446.04</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1.82795033658E9</v>
+        <v>1.82794731538E9</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>1.313754914E7</v>
+        <v>1.314057034E7</v>
       </c>
       <c r="L2" s="3">
         <f>D2-I2</f>
-        <v>58914.200000047684</v>
+        <v>61935.400000095367</v>
       </c>
       <c r="M2" s="3">
         <f>J2-E2</f>
-        <v>58914.199999999255</v>
+        <v>61935.400000000373</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
@@ -597,27 +597,27 @@
         <v>1.001119788E7</v>
       </c>
       <c r="F3" s="3">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G3" s="3">
         <v>100</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>60928.34</v>
+        <v>63949.58</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1.6840511172E8</v>
+        <v>1.6840209042E8</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>1.007212618E7</v>
+        <v>1.007514748E7</v>
       </c>
       <c r="L3" s="3">
         <f>D3-I3</f>
-        <v>59417.700000017881</v>
+        <v>62439</v>
       </c>
       <c r="M3" s="3">
         <f>J3-E3</f>
-        <v>59417.699999999255</v>
+        <v>62439</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.25">
@@ -637,27 +637,27 @@
         <v>9093507.28</v>
       </c>
       <c r="F4" s="3">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="G4" s="3">
         <v>100</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>61431.88</v>
+        <v>64453.12</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.03300365488E9</v>
+        <v>1.03300063368E9</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>9154939.18</v>
+        <v>9157960.38</v>
       </c>
       <c r="L4" s="3">
         <f>D4-I4</f>
-        <v>59921.299999952316</v>
+        <v>62942.5</v>
       </c>
       <c r="M4" s="3">
         <f>J4-E4</f>
-        <v>59921.300000000745</v>
+        <v>62942.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bidding completed for NAFED Gujrat Nccf
</commit_message>
<xml_diff>
--- a/testdata/BidDetailsData.xlsx.xlsx
+++ b/testdata/BidDetailsData.xlsx.xlsx
@@ -534,27 +534,27 @@
         <v>1.307712434E7</v>
       </c>
       <c r="F2" s="3">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="G2" s="3">
         <v>100</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>63446.04</v>
+        <v>50354.0</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1.82794731538E9</v>
+        <v>1.82796040738E9</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>1.314057034E7</v>
+        <v>1.312747834E7</v>
       </c>
       <c r="L2" s="3">
         <f>D2-I2</f>
-        <v>61935.400000095367</v>
+        <v>63446</v>
       </c>
       <c r="M2" s="3">
         <f>J2-E2</f>
-        <v>61935.400000000373</v>
+        <v>63446</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
@@ -597,27 +597,27 @@
         <v>1.001119788E7</v>
       </c>
       <c r="F3" s="3">
-        <v>127</v>
+        <v>101</v>
       </c>
       <c r="G3" s="3">
         <v>100</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>63949.58</v>
+        <v>50857.54</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1.6840209042E8</v>
+        <v>1.6841518252E8</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>1.007514748E7</v>
+        <v>1.006205538E7</v>
       </c>
       <c r="L3" s="3">
         <f>D3-I3</f>
-        <v>62439</v>
+        <v>63949.600000023842</v>
       </c>
       <c r="M3" s="3">
         <f>J3-E3</f>
-        <v>62439</v>
+        <v>63949.599999999627</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.25">
@@ -631,33 +631,33 @@
         <v>13</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.03306508678E9</v>
+        <v>1.03299358412E9</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>9093507.28</v>
+        <v>9157960.38</v>
       </c>
       <c r="F4" s="3">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="G4" s="3">
         <v>100</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>64453.12</v>
+        <v>51361.08</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.03300063368E9</v>
+        <v>1.03294222302E9</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>9157960.38</v>
+        <v>9209321.48</v>
       </c>
       <c r="L4" s="3">
         <f>D4-I4</f>
-        <v>62942.5</v>
+        <v>64453.100000023842</v>
       </c>
       <c r="M4" s="3">
         <f>J4-E4</f>
-        <v>62942.5</v>
+        <v>64453.10000000149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>